<commit_message>
CREI A V13!Dados de entrada ajustados! Metodologia inicialmente registrada como v3.
</commit_message>
<xml_diff>
--- a/input/Precos_Energia_por_Estado_v2 (2).xlsx
+++ b/input/Precos_Energia_por_Estado_v2 (2).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ead127730922d462/DOUTORADO/0.TESE/modelagem/steel_location_model/steel_location/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_34E3917B832CE937251A914307FA1C6C6CCEB162" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED426B6B-C150-4B2A-95AE-F1C9684EF632}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="11_34E3917B832CE937251A914307FA1C6C6CCEB162" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10049AE4-FB0E-4640-A741-08E4ACEE8A47}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="899" firstSheet="6" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="899" firstSheet="6" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LEIA-ME" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
     <sheet name="Ore_Cost_State" sheetId="16" r:id="rId16"/>
     <sheet name="Fuel_Prices_State" sheetId="17" r:id="rId17"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -2833,7 +2833,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2842,17 +2842,23 @@
     <col min="4" max="4" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="44" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="45" t="s">
+    <row r="2" spans="1:7" ht="66" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="62" t="s">
         <v>411</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+    </row>
+    <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="46" t="s">
         <v>126</v>
       </c>
@@ -2866,7 +2872,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="26" t="s">
         <v>221</v>
       </c>
@@ -2883,7 +2889,7 @@
         <v>37.298336284551112</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="26" t="s">
         <v>243</v>
       </c>
@@ -2900,7 +2906,7 @@
         <v>44.118186658027547</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="26" t="s">
         <v>273</v>
       </c>
@@ -2917,7 +2923,7 @@
         <v>50.302769079876775</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="26" t="s">
         <v>144</v>
       </c>
@@ -2934,7 +2940,7 @@
         <v>42.470299312238453</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="26" t="s">
         <v>197</v>
       </c>
@@ -2951,7 +2957,7 @@
         <v>41.275695537939697</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="26" t="s">
         <v>237</v>
       </c>
@@ -2968,7 +2974,7 @@
         <v>38.019990850661159</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="26" t="s">
         <v>262</v>
       </c>
@@ -2985,7 +2991,7 @@
         <v>47.569340726487574</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="26" t="s">
         <v>223</v>
       </c>
@@ -3002,7 +3008,7 @@
         <v>42.627099489945117</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="26" t="s">
         <v>193</v>
       </c>
@@ -3019,7 +3025,7 @@
         <v>39.4246144308526</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="26" t="s">
         <v>246</v>
       </c>
@@ -3036,7 +3042,7 @@
         <v>36.865836602327057</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="26" t="s">
         <v>158</v>
       </c>
@@ -3053,7 +3059,7 @@
         <v>43.569565106135599</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="26" t="s">
         <v>233</v>
       </c>
@@ -3335,6 +3341,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:G2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -3357,10 +3366,14 @@
         <v>416</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="45" t="s">
+    <row r="2" spans="1:6" ht="63" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="62" t="s">
         <v>417</v>
       </c>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="46" t="s">
@@ -3477,6 +3490,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -3499,7 +3515,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="62" t="s">
         <v>425</v>
       </c>
@@ -3672,10 +3688,13 @@
         <v>430</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="69.599999999999994" x14ac:dyDescent="0.3">
-      <c r="A2" s="45" t="s">
+    <row r="2" spans="1:5" ht="69.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="62" t="s">
         <v>431</v>
       </c>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
@@ -3922,6 +3941,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -3946,10 +3968,14 @@
         <v>446</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="45" t="s">
+    <row r="2" spans="1:8" ht="63" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="62" t="s">
         <v>447</v>
       </c>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="46" t="s">
@@ -4705,6 +4731,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -14677,7 +14706,7 @@
         <v>196.57</v>
       </c>
       <c r="G101" s="34">
-        <f t="shared" ref="G101:G132" si="9">E101+F101</f>
+        <f t="shared" ref="G101:G107" si="9">E101+F101</f>
         <v>293.26</v>
       </c>
       <c r="H101" s="33">
@@ -14687,7 +14716,7 @@
         <v>178.76</v>
       </c>
       <c r="J101" s="34">
-        <f t="shared" ref="J101:J132" si="10">H101+I101</f>
+        <f t="shared" ref="J101:J107" si="10">H101+I101</f>
         <v>258.52999999999997</v>
       </c>
       <c r="K101" s="33">
@@ -14697,7 +14726,7 @@
         <v>204.96</v>
       </c>
       <c r="M101" s="34">
-        <f t="shared" ref="M101:M132" si="11">K101+L101</f>
+        <f t="shared" ref="M101:M107" si="11">K101+L101</f>
         <v>290.39</v>
       </c>
       <c r="N101" s="34">

</xml_diff>